<commit_message>
update 2026-09-27 13:23 (plan 2026-10)
</commit_message>
<xml_diff>
--- a/7215c039a2_plan_2026-10.xlsx
+++ b/7215c039a2_plan_2026-10.xlsx
@@ -709,14 +709,14 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>2300</v>
+        <v>2100</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>530</v>
+        <v>480</v>
       </c>
     </row>
     <row r="6">
@@ -751,14 +751,14 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>600</v>
+        <v>2200</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>140</v>
+        <v>510</v>
       </c>
     </row>
     <row r="8">
@@ -772,14 +772,14 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>210</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9">
@@ -793,14 +793,14 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
@@ -814,14 +814,14 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -877,14 +877,14 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14">
@@ -919,14 +919,14 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16">
@@ -940,14 +940,14 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17">
@@ -961,14 +961,14 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>14.0%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>1400</v>
+        <v>700</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>320</v>
+        <v>160</v>
       </c>
     </row>
     <row r="18">
@@ -1216,10 +1216,10 @@
         <v>4987</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>2300</v>
+        <v>2100</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>-2686.978723404256</v>
+        <v>-2886.978723404256</v>
       </c>
       <c r="E4" s="18" t="inlineStr">
         <is>
@@ -1258,10 +1258,10 @@
         <v>154</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>600</v>
+        <v>2200</v>
       </c>
       <c r="D6" s="19" t="n">
-        <v>445.5979574468085</v>
+        <v>2045.597957446809</v>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
@@ -1279,10 +1279,10 @@
         <v>2653</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>-1752.5416</v>
+        <v>-1952.5416</v>
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
@@ -1300,10 +1300,10 @@
         <v>745</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>-344.8797531914894</v>
+        <v>-444.8797531914894</v>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
@@ -1321,10 +1321,10 @@
         <v>74</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>126.0372765957447</v>
+        <v>26.03727659574467</v>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
@@ -1384,10 +1384,10 @@
         <v>414</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="D12" s="17" t="n">
-        <v>-164.4995370212766</v>
+        <v>-264.4995370212766</v>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
@@ -1426,10 +1426,10 @@
         <v>1816</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>-1416.037446808511</v>
+        <v>-1516.037446808511</v>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
@@ -1579,13 +1579,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="11" t="n">
-        <v>34800</v>
+        <v>26400</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>36779.25873827122</v>
+        <v>27901.50662903334</v>
       </c>
       <c r="D3" s="22" t="n">
-        <v>963220.7412617288</v>
+        <v>972098.4933709666</v>
       </c>
     </row>
     <row r="4">
@@ -1593,13 +1593,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="11" t="n">
-        <v>69600</v>
+        <v>52800</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>78223.0480742552</v>
+        <v>59341.62267702119</v>
       </c>
       <c r="D4" s="22" t="n">
-        <v>921776.9519257448</v>
+        <v>940658.3773229788</v>
       </c>
     </row>
     <row r="5">
@@ -1607,13 +1607,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="11" t="n">
-        <v>104400</v>
+        <v>79200</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>124922.9472415584</v>
+        <v>94769.13239014772</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>875077.0527584417</v>
+        <v>905230.8676098522</v>
       </c>
     </row>
     <row r="6">
@@ -1621,13 +1621,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="11" t="n">
-        <v>139200</v>
+        <v>105600</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>177545.5625279147</v>
+        <v>134689.7370901422</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>822454.4374720854</v>
+        <v>865310.2629098578</v>
       </c>
     </row>
     <row r="7">
@@ -1635,13 +1635,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="11" t="n">
-        <v>174000</v>
+        <v>132000</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>236842.0425835862</v>
+        <v>179673.2736840999</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>763157.9574164138</v>
+        <v>820326.7263159001</v>
       </c>
     </row>
     <row r="8">
@@ -1649,13 +1649,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="11" t="n">
-        <v>208800</v>
+        <v>158400</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>303658.8005090381</v>
+        <v>230361.8486620288</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>696341.1994909619</v>
+        <v>769638.1513379712</v>
       </c>
     </row>
     <row r="9">
@@ -1663,13 +1663,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>243600</v>
+        <v>184800</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>378949.5957717058</v>
+        <v>287479.0036888803</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>621050.4042282942</v>
+        <v>712520.9963111198</v>
       </c>
     </row>
     <row r="10">
@@ -1677,13 +1677,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="11" t="n">
-        <v>278400</v>
+        <v>211200</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>463789.1484122216</v>
+        <v>351840.0436230646</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>536210.8515877784</v>
+        <v>648159.9563769354</v>
       </c>
     </row>
     <row r="11">
@@ -1691,13 +1691,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="11" t="n">
-        <v>313200</v>
+        <v>237600</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>559388.4798727535</v>
+        <v>424363.6743862267</v>
       </c>
       <c r="D11" s="22" t="n">
-        <v>440611.5201272465</v>
+        <v>575636.3256137733</v>
       </c>
     </row>
     <row r="12">
@@ -1705,13 +1705,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="11" t="n">
-        <v>348000</v>
+        <v>264000</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>667112.1994263635</v>
+        <v>506085.1168062067</v>
       </c>
       <c r="D12" s="22" t="n">
-        <v>332887.8005736365</v>
+        <v>493914.8831937933</v>
       </c>
     </row>
     <row r="13">
@@ -1719,13 +1719,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="11" t="n">
-        <v>382800</v>
+        <v>290400</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>788497.9829582878</v>
+        <v>598170.8836235285</v>
       </c>
       <c r="D13" s="22" t="n">
-        <v>211502.0170417122</v>
+        <v>401829.1163764715</v>
       </c>
     </row>
     <row r="14">
@@ -1733,13 +1733,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="11" t="n">
-        <v>417600</v>
+        <v>316800</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>925278.5221442414</v>
+        <v>701935.4305921829</v>
       </c>
       <c r="D14" s="22" t="n">
-        <v>74721.47785575863</v>
+        <v>298064.5694078171</v>
       </c>
     </row>
     <row r="15">
@@ -1747,13 +1747,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="11" t="n">
-        <v>452400</v>
-      </c>
-      <c r="C15" s="9" t="n">
-        <v>1079406.25733392</v>
-      </c>
-      <c r="D15" s="23" t="n">
-        <v>0</v>
+        <v>343200</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>818859.919356767</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>181140.080643233</v>
       </c>
     </row>
     <row r="16">
@@ -1761,13 +1761,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="11" t="n">
-        <v>487200</v>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v>1253081.247183203</v>
-      </c>
-      <c r="D16" s="23" t="n">
-        <v>0</v>
+        <v>369600</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>950613.3599320849</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>49386.64006791508</v>
       </c>
     </row>
     <row r="17">
@@ -1775,10 +1775,10 @@
         <v>15</v>
       </c>
       <c r="B17" s="11" t="n">
-        <v>522000</v>
+        <v>396000</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>1448782.572853291</v>
+        <v>1099076.434578358</v>
       </c>
       <c r="D17" s="23" t="n">
         <v>0</v>

</xml_diff>